<commit_message>
update accuracy object detection
</commit_message>
<xml_diff>
--- a/accuracy.xlsx
+++ b/accuracy.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="24">
   <si>
     <t>YOLOV8</t>
   </si>
@@ -629,7 +629,7 @@
         <v>106</v>
       </c>
       <c r="D3" s="6">
-        <f>(C3/B3)</f>
+        <f t="shared" ref="D3:D16" si="0">(C3/B3)</f>
         <v>0.95495495495495497</v>
       </c>
       <c r="E3" s="1"/>
@@ -652,7 +652,7 @@
         <v>51</v>
       </c>
       <c r="D4" s="9">
-        <f>(C4/B4)</f>
+        <f t="shared" si="0"/>
         <v>0.85</v>
       </c>
       <c r="E4" s="1"/>
@@ -675,7 +675,7 @@
         <v>98</v>
       </c>
       <c r="D5" s="7">
-        <f>(C5/B5)</f>
+        <f t="shared" si="0"/>
         <v>0.81666666666666665</v>
       </c>
       <c r="E5" s="1"/>
@@ -698,7 +698,7 @@
         <v>194</v>
       </c>
       <c r="D6" s="7">
-        <f>(C6/B6)</f>
+        <f t="shared" si="0"/>
         <v>0.99487179487179489</v>
       </c>
       <c r="E6" s="1"/>
@@ -721,7 +721,7 @@
         <v>168</v>
       </c>
       <c r="D7" s="7">
-        <f>(C7/B7)</f>
+        <f t="shared" si="0"/>
         <v>0.96551724137931039</v>
       </c>
       <c r="E7" s="1"/>
@@ -744,7 +744,7 @@
         <v>96</v>
       </c>
       <c r="D8" s="9">
-        <f>(C8/B8)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E8" s="1"/>
@@ -767,7 +767,7 @@
         <v>172</v>
       </c>
       <c r="D9" s="9">
-        <f>(C9/B9)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E9" s="1"/>
@@ -790,7 +790,7 @@
         <v>158</v>
       </c>
       <c r="D10" s="7">
-        <f>(C10/B10)</f>
+        <f t="shared" si="0"/>
         <v>0.95757575757575752</v>
       </c>
       <c r="E10" s="1"/>
@@ -813,7 +813,7 @@
         <v>116</v>
       </c>
       <c r="D11" s="7">
-        <f>(C11/B11)</f>
+        <f t="shared" si="0"/>
         <v>0.77333333333333332</v>
       </c>
       <c r="E11" s="1"/>
@@ -836,7 +836,7 @@
         <v>143</v>
       </c>
       <c r="D12" s="7">
-        <f>(C12/B12)</f>
+        <f t="shared" si="0"/>
         <v>0.99305555555555558</v>
       </c>
       <c r="E12" s="1"/>
@@ -859,7 +859,7 @@
         <v>177</v>
       </c>
       <c r="D13" s="9">
-        <f>(C13/B13)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E13" s="1"/>
@@ -882,7 +882,7 @@
         <v>82</v>
       </c>
       <c r="D14" s="7">
-        <f>(C14/B14)</f>
+        <f t="shared" si="0"/>
         <v>0.97619047619047616</v>
       </c>
       <c r="E14" s="1"/>
@@ -905,7 +905,7 @@
         <v>103</v>
       </c>
       <c r="D15" s="7">
-        <f>(C15/B15)</f>
+        <f t="shared" si="0"/>
         <v>0.99038461538461542</v>
       </c>
       <c r="E15" s="1"/>
@@ -928,7 +928,7 @@
         <v>139</v>
       </c>
       <c r="D16" s="7">
-        <f>(C16/B16)</f>
+        <f t="shared" si="0"/>
         <v>0.95205479452054798</v>
       </c>
       <c r="E16" s="1"/>
@@ -1026,10 +1026,20 @@
         <f>(C21/B21)</f>
         <v>0.99099099099099097</v>
       </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="E21" s="1">
+        <v>111</v>
+      </c>
+      <c r="F21" s="9">
+        <f>(E21/B21)</f>
+        <v>1</v>
+      </c>
+      <c r="G21" s="1">
+        <v>110</v>
+      </c>
+      <c r="H21" s="7">
+        <f>G21/B21</f>
+        <v>0.99099099099099097</v>
+      </c>
       <c r="I21" s="12"/>
       <c r="J21" s="13"/>
       <c r="K21" s="13"/>
@@ -1046,13 +1056,23 @@
         <v>50</v>
       </c>
       <c r="D22" s="7">
-        <f>(C22/B22)</f>
+        <f t="shared" ref="D21:D34" si="1">(C22/B22)</f>
         <v>0.83333333333333337</v>
       </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="E22" s="1">
+        <v>51</v>
+      </c>
+      <c r="F22" s="9">
+        <f t="shared" ref="F22:F34" si="2">(E22/B22)</f>
+        <v>0.85</v>
+      </c>
+      <c r="G22" s="1">
+        <v>53</v>
+      </c>
+      <c r="H22" s="7">
+        <f t="shared" ref="H22:H34" si="3">G22/B22</f>
+        <v>0.8833333333333333</v>
+      </c>
       <c r="I22" s="12"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
@@ -1069,13 +1089,23 @@
         <v>106</v>
       </c>
       <c r="D23" s="7">
-        <f>(C23/B23)</f>
+        <f t="shared" si="1"/>
         <v>0.8833333333333333</v>
       </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
+      <c r="E23" s="1">
+        <v>105</v>
+      </c>
+      <c r="F23" s="7">
+        <f t="shared" si="2"/>
+        <v>0.875</v>
+      </c>
+      <c r="G23" s="1">
+        <v>105</v>
+      </c>
+      <c r="H23" s="7">
+        <f t="shared" si="3"/>
+        <v>0.875</v>
+      </c>
       <c r="I23" s="12"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
@@ -1092,13 +1122,23 @@
         <v>195</v>
       </c>
       <c r="D24" s="9">
-        <f>(C24/B24)</f>
-        <v>1</v>
-      </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E24" s="1">
+        <v>195</v>
+      </c>
+      <c r="F24" s="9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="G24" s="1">
+        <v>194</v>
+      </c>
+      <c r="H24" s="7">
+        <f t="shared" si="3"/>
+        <v>0.99487179487179489</v>
+      </c>
       <c r="I24" s="12"/>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
@@ -1115,13 +1155,23 @@
         <v>168</v>
       </c>
       <c r="D25" s="7">
-        <f>(C25/B25)</f>
+        <f t="shared" si="1"/>
         <v>0.96551724137931039</v>
       </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
+      <c r="E25" s="1">
+        <v>167</v>
+      </c>
+      <c r="F25" s="7">
+        <f t="shared" si="2"/>
+        <v>0.95977011494252873</v>
+      </c>
+      <c r="G25" s="1">
+        <v>167</v>
+      </c>
+      <c r="H25" s="7">
+        <f t="shared" si="3"/>
+        <v>0.95977011494252873</v>
+      </c>
       <c r="I25" s="12"/>
       <c r="J25" s="13"/>
       <c r="K25" s="13"/>
@@ -1138,13 +1188,23 @@
         <v>96</v>
       </c>
       <c r="D26" s="9">
-        <f>(C26/B26)</f>
-        <v>1</v>
-      </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E26" s="1">
+        <v>96</v>
+      </c>
+      <c r="F26" s="9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="G26" s="1">
+        <v>96</v>
+      </c>
+      <c r="H26" s="9">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
       <c r="I26" s="12"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
@@ -1161,13 +1221,23 @@
         <v>172</v>
       </c>
       <c r="D27" s="9">
-        <f>(C27/B27)</f>
-        <v>1</v>
-      </c>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E27" s="1">
+        <v>172</v>
+      </c>
+      <c r="F27" s="9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="G27" s="1">
+        <v>172</v>
+      </c>
+      <c r="H27" s="9">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
       <c r="I27" s="12"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
@@ -1184,13 +1254,23 @@
         <v>154</v>
       </c>
       <c r="D28" s="7">
-        <f>(C28/B28)</f>
+        <f t="shared" si="1"/>
         <v>0.93333333333333335</v>
       </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
+      <c r="E28" s="1">
+        <v>154</v>
+      </c>
+      <c r="F28" s="7">
+        <f t="shared" si="2"/>
+        <v>0.93333333333333335</v>
+      </c>
+      <c r="G28" s="1">
+        <v>155</v>
+      </c>
+      <c r="H28" s="7">
+        <f t="shared" si="3"/>
+        <v>0.93939393939393945</v>
+      </c>
       <c r="I28" s="12"/>
       <c r="J28" s="13"/>
       <c r="K28" s="13"/>
@@ -1207,13 +1287,23 @@
         <v>141</v>
       </c>
       <c r="D29" s="9">
-        <f>(C29/B29)</f>
+        <f t="shared" si="1"/>
         <v>0.94</v>
       </c>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
+      <c r="E29" s="1">
+        <v>139</v>
+      </c>
+      <c r="F29" s="7">
+        <f t="shared" si="2"/>
+        <v>0.92666666666666664</v>
+      </c>
+      <c r="G29" s="1">
+        <v>143</v>
+      </c>
+      <c r="H29" s="7">
+        <f t="shared" si="3"/>
+        <v>0.95333333333333337</v>
+      </c>
       <c r="I29" s="12"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13"/>
@@ -1230,13 +1320,23 @@
         <v>143</v>
       </c>
       <c r="D30" s="7">
-        <f>(C30/B30)</f>
+        <f t="shared" si="1"/>
         <v>0.99305555555555558</v>
       </c>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
+      <c r="E30" s="1">
+        <v>144</v>
+      </c>
+      <c r="F30" s="9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="G30" s="1">
+        <v>143</v>
+      </c>
+      <c r="H30" s="7">
+        <f t="shared" si="3"/>
+        <v>0.99305555555555558</v>
+      </c>
       <c r="I30" s="12"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
@@ -1253,13 +1353,23 @@
         <v>177</v>
       </c>
       <c r="D31" s="9">
-        <f>(C31/B31)</f>
-        <v>1</v>
-      </c>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E31" s="1">
+        <v>176</v>
+      </c>
+      <c r="F31" s="7">
+        <f t="shared" si="2"/>
+        <v>0.99435028248587576</v>
+      </c>
+      <c r="G31" s="1">
+        <v>177</v>
+      </c>
+      <c r="H31" s="9">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
       <c r="I31" s="12"/>
       <c r="J31" s="13"/>
       <c r="K31" s="13"/>
@@ -1276,13 +1386,23 @@
         <v>83</v>
       </c>
       <c r="D32" s="7">
-        <f>(C32/B32)</f>
+        <f t="shared" si="1"/>
         <v>0.98809523809523814</v>
       </c>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
+      <c r="E32" s="1">
+        <v>83</v>
+      </c>
+      <c r="F32" s="7">
+        <f t="shared" si="2"/>
+        <v>0.98809523809523814</v>
+      </c>
+      <c r="G32" s="1">
+        <v>82</v>
+      </c>
+      <c r="H32" s="7">
+        <f t="shared" si="3"/>
+        <v>0.97619047619047616</v>
+      </c>
       <c r="I32" s="12"/>
       <c r="J32" s="13"/>
       <c r="K32" s="13"/>
@@ -1299,13 +1419,23 @@
         <v>103</v>
       </c>
       <c r="D33" s="7">
-        <f>(C33/B33)</f>
+        <f t="shared" si="1"/>
         <v>0.99038461538461542</v>
       </c>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
+      <c r="E33" s="1">
+        <v>104</v>
+      </c>
+      <c r="F33" s="9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="G33" s="1">
+        <v>103</v>
+      </c>
+      <c r="H33" s="7">
+        <f t="shared" si="3"/>
+        <v>0.99038461538461542</v>
+      </c>
       <c r="I33" s="12"/>
       <c r="J33" s="13"/>
       <c r="K33" s="13"/>
@@ -1322,13 +1452,23 @@
         <v>139</v>
       </c>
       <c r="D34" s="7">
-        <f>(C34/B34)</f>
+        <f t="shared" si="1"/>
         <v>0.95205479452054798</v>
       </c>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
+      <c r="E34" s="1">
+        <v>140</v>
+      </c>
+      <c r="F34" s="7">
+        <f t="shared" si="2"/>
+        <v>0.95890410958904104</v>
+      </c>
+      <c r="G34" s="1">
+        <v>138</v>
+      </c>
+      <c r="H34" s="7">
+        <f t="shared" si="3"/>
+        <v>0.9452054794520548</v>
+      </c>
       <c r="I34" s="12"/>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -1344,10 +1484,20 @@
         <f>SUM(C21:C34)/SUM(B21:B34)</f>
         <v>0.96786090621707055</v>
       </c>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
+      <c r="E35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="7">
+        <f>SUM(E21:E34)/SUM(B21:B34)</f>
+        <v>0.96786090621707055</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="7">
+        <f>SUM(G21:G34)/SUM(B21:B34)</f>
+        <v>0.96838777660695474</v>
+      </c>
       <c r="I35" s="12"/>
       <c r="J35" s="13"/>
       <c r="K35" s="13"/>

</xml_diff>